<commit_message>
Cards: bat/bats are baseball bats, not the animal
New card art for card_bat/card_bats (assets/card) and the game copies in card_web. Korean label 박쥐 → 야구방망이 (개) in build_words.py, words.js and the word list. ?v=2 on the bat/bats entries in cards.js and on its script tag, so browsers that cached the old bat on the share link fetch the new one.
</commit_message>
<xml_diff>
--- a/카드_낱말_목록.xlsx
+++ b/카드_낱말_목록.xlsx
@@ -808,12 +808,12 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>박쥐 한 마리</t>
+          <t>야구방망이 한 개</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>박쥐 여러 마리</t>
+          <t>야구방망이 여러 개</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
@@ -1892,12 +1892,12 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>박쥐 한 마리</t>
+          <t>야구방망이 한 개</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>박쥐 여러 마리</t>
+          <t>야구방망이 여러 개</t>
         </is>
       </c>
       <c r="F19" s="4" t="n">

</xml_diff>